<commit_message>
Added application preview test. Added php script to connect to mySQL database.
</commit_message>
<xml_diff>
--- a/Doc/PropertiesList.xlsx
+++ b/Doc/PropertiesList.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t xml:space="preserve">Elements for table "PropertiesList"</t>
   </si>
@@ -34,25 +34,28 @@
     <t xml:space="preserve">INT (AUTO_INCREMENT PRIMARY KEY)</t>
   </si>
   <si>
-    <t xml:space="preserve">original_price</t>
+    <t xml:space="preserve">price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLOAT UNSIGNED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">number_of_rooms</t>
   </si>
   <si>
     <t xml:space="preserve">INT</t>
   </si>
   <si>
-    <t xml:space="preserve">current_price</t>
-  </si>
-  <si>
-    <t xml:space="preserve">number_of_rooms</t>
-  </si>
-  <si>
     <t xml:space="preserve">number_of_bathrooms</t>
   </si>
   <si>
     <t xml:space="preserve">area_sqft</t>
   </si>
   <si>
-    <t xml:space="preserve">address_number</t>
+    <t xml:space="preserve">property_state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TINYINT </t>
   </si>
   <si>
     <t xml:space="preserve">address_street</t>
@@ -61,6 +64,12 @@
     <t xml:space="preserve">VARCHAR(50)</t>
   </si>
   <si>
+    <t xml:space="preserve">address_apartment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VARCHAR(10)</t>
+  </si>
+  <si>
     <t xml:space="preserve">address_city</t>
   </si>
   <si>
@@ -70,46 +79,10 @@
     <t xml:space="preserve">address_zip</t>
   </si>
   <si>
-    <t xml:space="preserve">for_sale</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BOOLEAN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">for_rent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">for_sale_by</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(owner or realtor)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">garage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">garage_spot_number</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pool</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hoa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">monthly_hoa_cost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TEXT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">favorite</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BOOLEAN (default false?)</t>
+    <t xml:space="preserve">MEDIUMINT UNSIGNED</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -204,15 +177,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -233,134 +206,122 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Z22"/>
+  <dimension ref="A1:Z26"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="40.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="36.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="40.12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="1" t="s">
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
+      <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
+      <c r="B7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="1" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="B8" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>12</v>
-      </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>12</v>
+      <c r="A11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>5</v>
+      <c r="A12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>17</v>
-      </c>
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>17</v>
-      </c>
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>20</v>
-      </c>
+      <c r="A15" s="3"/>
+      <c r="B15" s="3"/>
       <c r="C15" s="3"/>
-      <c r="D15" s="2"/>
+      <c r="D15" s="3"/>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
@@ -384,60 +345,37 @@
       <c r="Y15" s="3"/>
       <c r="Z15" s="3"/>
     </row>
-    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>29</v>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+    </row>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+    </row>
+    <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>